<commit_message>
fix: add exa-py dep, fix dead Swiss URLs, limit Tandem to one search
- requirements.txt: add exa-py>=1.0.0 (was silently skipped in CI)
- _registry.py: skip 4 companies with dead/moved domains (AlloCyte,
  PharmaBiome, Stromal Therapeutics, SYDRA AG); update 3 URLs
  (Basilea, PSI CRO, Opna Bio); add keywords_override field to
  SiteConfig so per-site keyword lists can be set
- Tandem Therapeutics: keywords_override=["chemist"] — Ashby board
  ignores the search param and returns all jobs every time; scraping
  once with a broad term cuts noise from 160 to ~20 jobs
- _coordinator.py: _effective_keywords honours keywords_override
- European_Job_Search_Websites.xlsx: updated 3 URLs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/European_Job_Search_Websites.xlsx
+++ b/European_Job_Search_Websites.xlsx
@@ -2813,7 +2813,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://jobs.basilea.com/eng</t>
+          <t>https://www.basilea.com/careers</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3715,7 +3715,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>https://psicro.com/careers/</t>
+          <t>https://psi-cro.com/careers/</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>https://opnabio.com/careers/</t>
+          <t>https://www.opnabio.com/careers/</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">

</xml_diff>

<commit_message>
feat: add Status column to company Excel, remove SpiroChem
- European_Job_Search_Websites.xlsx: new Status column (Active/Skip,
  colour-coded) lets users toggle companies without touching code;
  SpiroChem row removed
- _registry.py: load_sites() reads Status column — "Skip" in the
  spreadsheet marks a site inactive; _OVERRIDES technical skips
  (login-walls, big pharma, dead domains) still take precedence;
  SpiroChem override removed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/European_Job_Search_Websites.xlsx
+++ b/European_Job_Search_Websites.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +48,11 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +67,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -93,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -115,6 +130,13 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -481,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D164"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -511,6 +533,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -533,6 +560,11 @@
           <t>Austria's largest general job board</t>
         </is>
       </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -555,6 +587,11 @@
           <t>Strong for professional and corporate roles</t>
         </is>
       </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -577,6 +614,11 @@
           <t>Flemish public employment service</t>
         </is>
       </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -599,6 +641,11 @@
           <t>Major generalist job board</t>
         </is>
       </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -621,6 +668,11 @@
           <t>Walloon public employment service</t>
         </is>
       </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -643,6 +695,11 @@
           <t>Denmark's largest job portal</t>
         </is>
       </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -665,6 +722,11 @@
           <t>Official portal for international job seekers</t>
         </is>
       </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -687,6 +749,11 @@
           <t>Official public employment service</t>
         </is>
       </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -709,6 +776,11 @@
           <t>Leading private job board</t>
         </is>
       </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -731,6 +803,11 @@
           <t>Popular job aggregator</t>
         </is>
       </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -753,6 +830,11 @@
           <t>Largest job aggregator in France</t>
         </is>
       </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -775,6 +857,11 @@
           <t>Official public employment service (formerly Pôle Emploi)</t>
         </is>
       </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -797,6 +884,11 @@
           <t>Specialized for managers and executives</t>
         </is>
       </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -819,6 +911,11 @@
           <t>Leading professional job board</t>
         </is>
       </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -841,6 +938,11 @@
           <t>Highest traffic job aggregator</t>
         </is>
       </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -863,6 +965,11 @@
           <t>Federal Employment Agency job portal</t>
         </is>
       </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -885,6 +992,11 @@
           <t>Germany's LinkedIn alternative for DACH region</t>
         </is>
       </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -907,6 +1019,11 @@
           <t>One of Ireland's largest job sites</t>
         </is>
       </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -929,6 +1046,11 @@
           <t>Major Irish generalist job board</t>
         </is>
       </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -951,6 +1073,11 @@
           <t>Widely used aggregator in Ireland</t>
         </is>
       </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -973,6 +1100,11 @@
           <t>Top generalist job board</t>
         </is>
       </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -995,6 +1127,11 @@
           <t>Major job aggregator</t>
         </is>
       </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1017,6 +1154,11 @@
           <t>International board with strong Italian presence</t>
         </is>
       </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1039,6 +1181,11 @@
           <t>Leading job aggregator</t>
         </is>
       </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1061,6 +1208,11 @@
           <t>Major Dutch job board</t>
         </is>
       </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1083,6 +1235,11 @@
           <t>UWV official government job portal</t>
         </is>
       </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1105,6 +1262,11 @@
           <t>~80% market share, Norway's dominant job board</t>
         </is>
       </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1127,6 +1289,11 @@
           <t>Official public employment portal</t>
         </is>
       </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1149,6 +1316,11 @@
           <t>Strong for academic and public sector jobs</t>
         </is>
       </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1171,6 +1343,11 @@
           <t>Poland's largest job board</t>
         </is>
       </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1193,6 +1370,11 @@
           <t>Major general job platform</t>
         </is>
       </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1215,6 +1397,11 @@
           <t>Top IT and tech job board</t>
         </is>
       </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1237,6 +1424,11 @@
           <t>Major national job board</t>
         </is>
       </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -1259,6 +1451,11 @@
           <t>Popular local job portal</t>
         </is>
       </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1281,6 +1478,11 @@
           <t>Strong for tech jobs, based in Portugal</t>
         </is>
       </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1303,6 +1505,11 @@
           <t>Spain's #1 job board</t>
         </is>
       </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1325,6 +1532,11 @@
           <t>Major generalist job board</t>
         </is>
       </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1347,6 +1559,11 @@
           <t>Strong job aggregator</t>
         </is>
       </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -1369,6 +1586,11 @@
           <t>Official public employment service</t>
         </is>
       </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -1391,6 +1613,11 @@
           <t>Leading job aggregator</t>
         </is>
       </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -1413,6 +1640,11 @@
           <t>Popular aggregator with ~55,000 listings</t>
         </is>
       </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1435,6 +1667,11 @@
           <t>#1 portal, strong in German-speaking regions</t>
         </is>
       </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1457,6 +1694,11 @@
           <t>Leader in French-speaking Romandie</t>
         </is>
       </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1479,6 +1721,11 @@
           <t>Broad national Swiss job board</t>
         </is>
       </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1501,6 +1748,11 @@
           <t>Official public employment service</t>
         </is>
       </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -1523,6 +1775,11 @@
           <t>UK's #1 job site</t>
         </is>
       </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -1545,6 +1802,11 @@
           <t>Leading UK-focused job board</t>
         </is>
       </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -1567,6 +1829,11 @@
           <t>Major generalist UK platform</t>
         </is>
       </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1589,6 +1856,11 @@
           <t>Official EU portal, ~3M jobs across 31 countries</t>
         </is>
       </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1611,6 +1883,11 @@
           <t>Strong across all of Western Europe</t>
         </is>
       </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1633,6 +1910,11 @@
           <t>Job listings combined with company reviews</t>
         </is>
       </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1655,6 +1937,11 @@
           <t>Pharma; Basel HQ</t>
         </is>
       </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1677,6 +1964,11 @@
           <t>Pharma; Basel office</t>
         </is>
       </c>
+      <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1699,6 +1991,11 @@
           <t>Pharma; Basel HQ</t>
         </is>
       </c>
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1721,6 +2018,11 @@
           <t>Pharma; Basel HQ</t>
         </is>
       </c>
+      <c r="E56" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1743,6 +2045,11 @@
           <t>Pharma generics; Basel</t>
         </is>
       </c>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1765,6 +2072,11 @@
           <t>Pharma; Basel &amp; Vernier</t>
         </is>
       </c>
+      <c r="E58" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1787,6 +2099,11 @@
           <t>Pharma; Basel hub</t>
         </is>
       </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1809,6 +2126,11 @@
           <t>Pharma; European HQ Basel (Workday)</t>
         </is>
       </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1831,6 +2153,11 @@
           <t>Pharma; mRNA; Basel hub</t>
         </is>
       </c>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1853,6 +2180,11 @@
           <t>Pharma generics; Basel</t>
         </is>
       </c>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1875,6 +2207,11 @@
           <t>Specialty biochemicals; Basel</t>
         </is>
       </c>
+      <c r="E63" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1897,6 +2234,11 @@
           <t>Pharma SOBI; Basel (Cornerstone)</t>
         </is>
       </c>
+      <c r="E64" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1919,6 +2261,11 @@
           <t>CDMO; Basel HQ</t>
         </is>
       </c>
+      <c r="E65" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1941,6 +2288,11 @@
           <t>Biologics CDMO; Basel (Personio)</t>
         </is>
       </c>
+      <c r="E66" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1963,6 +2315,11 @@
           <t>Lyophilisation CDMO; Basel</t>
         </is>
       </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1985,6 +2342,11 @@
           <t>Drug dev CDMO; Basel</t>
         </is>
       </c>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1994,17 +2356,22 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SpiroChem</t>
+          <t>Bright Peak Therapeutics</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://spirochem.com/careers/</t>
+          <t>https://jobs.ashbyhq.com/brightpeak</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Discovery CRO; Basel</t>
+          <t>Biotech; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2016,17 +2383,22 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Bright Peak Therapeutics</t>
+          <t>BioVersys</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/brightpeak</t>
+          <t>https://www.bioversys.com/careers/</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Biotech; Basel (Ashby)</t>
+          <t>Biotech antibiotics; Basel</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2038,17 +2410,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>BioVersys</t>
+          <t>Noema Pharma</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://www.bioversys.com/careers/</t>
+          <t>https://jobs.ashbyhq.com/noema</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Biotech antibiotics; Basel</t>
+          <t>Biotech CNS; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2060,17 +2437,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Noema Pharma</t>
+          <t>Monte Rosa Therapeutics</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/noema</t>
+          <t>https://jobs.ashbyhq.com/MonteRosaTherapeutics</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Biotech CNS; Basel (Ashby)</t>
+          <t>Biotech molecular glue; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2082,17 +2464,22 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Monte Rosa Therapeutics</t>
+          <t>NBE-Therapeutics</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/MonteRosaTherapeutics</t>
+          <t>https://nbe-therapeutics.com/employment/vacancies/</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Biotech molecular glue; Basel (Ashby)</t>
+          <t>Biotech ADC; Basel</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2104,17 +2491,22 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>NBE-Therapeutics</t>
+          <t>Vir Biotechnology</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://nbe-therapeutics.com/employment/vacancies/</t>
+          <t>https://jobs.ashbyhq.com/vir</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Biotech ADC; Basel</t>
+          <t>Biotech infectious disease; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2126,17 +2518,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Vir Biotechnology</t>
+          <t>Roivant Sciences</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/vir</t>
+          <t>https://jobs.ashbyhq.com/roivant</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Biotech infectious disease; Basel (Ashby)</t>
+          <t>Biotech; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2148,17 +2545,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Roivant Sciences</t>
+          <t>FoRx Therapeutics</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/roivant</t>
+          <t>https://www.forxtherapeutics.com/career</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Biotech; Basel (Ashby)</t>
+          <t>Biotech; Basel</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2170,17 +2572,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>FoRx Therapeutics</t>
+          <t>Cimeio Therapeutics</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://www.forxtherapeutics.com/career</t>
+          <t>https://www.cimeio.com/careers/</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Biotech; Basel</t>
+          <t>Biotech cell &amp; gene; Basel</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2192,17 +2599,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Cimeio Therapeutics</t>
+          <t>Mosanna Therapeutics</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://www.cimeio.com/careers/</t>
+          <t>https://mosanna.com/careers/</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Biotech cell &amp; gene; Basel</t>
+          <t>Biotech; Basel</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2214,17 +2626,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Mosanna Therapeutics</t>
+          <t>Synendos Therapeutics</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://mosanna.com/careers/</t>
+          <t>https://www.synendos.com/open-position</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Biotech; Basel</t>
+          <t>Biotech endocannabinoid; Basel</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2236,17 +2653,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Synendos Therapeutics</t>
+          <t>Tolremo Therapeutics</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://www.synendos.com/open-position</t>
+          <t>https://www.tolremo.com/careers</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Biotech endocannabinoid; Basel</t>
+          <t>Biotech; Basel</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2258,17 +2680,22 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Tolremo Therapeutics</t>
+          <t>Vaximm</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://www.tolremo.com/careers</t>
+          <t>https://vaximm.com/about-us/</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Biotech; Basel</t>
+          <t>Biotech oral vaccines; Basel</t>
+        </is>
+      </c>
+      <c r="E81" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2280,17 +2707,22 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Vaximm</t>
+          <t>Versameb</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://vaximm.com/about-us/</t>
+          <t>https://versameb.com/contact/career/</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Biotech oral vaccines; Basel</t>
+          <t>Biotech mRNA; Basel</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2302,17 +2734,22 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Versameb</t>
+          <t>Genedata</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://versameb.com/contact/career/</t>
+          <t>https://jobs.danaher.com/global/en/genedata</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Biotech mRNA; Basel</t>
+          <t>Bioinfo software; Basel (Danaher)</t>
+        </is>
+      </c>
+      <c r="E83" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2324,17 +2761,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Genedata</t>
+          <t>Scailyte</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://jobs.danaher.com/global/en/genedata</t>
+          <t>https://scailyte.com/careers/</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Bioinfo software; Basel (Danaher)</t>
+          <t>Biotech single-cell AI; Basel</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2346,17 +2788,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Scailyte</t>
+          <t>Oxford BioTherapeutics</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://scailyte.com/careers/</t>
+          <t>https://www.oxfordbiotherapeutics.com/careers</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Biotech single-cell AI; Basel</t>
+          <t>Biotech ADC oncology; Basel</t>
+        </is>
+      </c>
+      <c r="E85" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2368,17 +2815,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Oxford BioTherapeutics</t>
+          <t>Skyhawk Therapeutics</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://www.oxfordbiotherapeutics.com/careers</t>
+          <t>https://job-boards.greenhouse.io/skyhawktherapeutics</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Biotech ADC oncology; Basel</t>
+          <t>Biotech RNA splicing; Basel (Greenhouse)</t>
+        </is>
+      </c>
+      <c r="E86" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2390,17 +2842,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Skyhawk Therapeutics</t>
+          <t>Alentis Therapeutics</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/skyhawktherapeutics</t>
+          <t>https://jobs.ashbyhq.com/alentis</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Biotech RNA splicing; Basel (Greenhouse)</t>
+          <t>Biotech fibrosis &amp; cancer; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2412,17 +2869,22 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Alentis Therapeutics</t>
+          <t>Windward Bio</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/alentis</t>
+          <t>https://jobs.ashbyhq.com/WindwardBio</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Biotech fibrosis &amp; cancer; Basel (Ashby)</t>
+          <t>Biotech immunology; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2434,17 +2896,22 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Windward Bio</t>
+          <t>Anaveon</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/WindwardBio</t>
+          <t>https://anaveon.com/careers/</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Biotech immunology; Basel (Ashby)</t>
+          <t>Biotech IL-2; Basel</t>
+        </is>
+      </c>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2456,17 +2923,22 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Anaveon</t>
+          <t>RhyGaze</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://anaveon.com/careers/</t>
+          <t>https://rhygaze.com/careers/</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Biotech IL-2; Basel</t>
+          <t>Biotech gene therapy; Basel</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2478,17 +2950,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>RhyGaze</t>
+          <t>Captor Therapeutics</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://rhygaze.com/careers/</t>
+          <t>https://jobs.ashbyhq.com/captor</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Biotech gene therapy; Basel</t>
+          <t>Biotech molecular glue; Basel (Ashby)</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2500,17 +2977,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Captor Therapeutics</t>
+          <t>Altamira Therapeutics</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/captor</t>
+          <t>https://www.altamiratherapeutics.com/careers/</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Biotech molecular glue; Basel (Ashby)</t>
+          <t>Biotech RNA delivery; Basel</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2522,17 +3004,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Altamira Therapeutics</t>
+          <t>Alloy Therapeutics</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://www.altamiratherapeutics.com/careers/</t>
+          <t>https://www.alloytx.com/careers/</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Biotech RNA delivery; Basel</t>
+          <t>Biotech antibody; Basel</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2544,17 +3031,22 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Alloy Therapeutics</t>
+          <t>Amporin Pharmaceuticals</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://www.alloytx.com/careers/</t>
+          <t>https://amporin.com/careers/</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Biotech antibody; Basel</t>
+          <t>Biotech small molecules; Basel</t>
+        </is>
+      </c>
+      <c r="E94" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2566,17 +3058,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Amporin Pharmaceuticals</t>
+          <t>AlloCyte Pharmaceuticals</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://amporin.com/careers/</t>
+          <t>https://allocyte.com/careers/</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Biotech small molecules; Basel</t>
+          <t>Biotech allogeneic cell; Basel</t>
+        </is>
+      </c>
+      <c r="E95" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -2588,17 +3085,22 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>AlloCyte Pharmaceuticals</t>
+          <t>Ridgeline Discovery</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://allocyte.com/careers/</t>
+          <t>https://ridgelinediscovery.com/careers/</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Biotech allogeneic cell; Basel</t>
+          <t>CRO drug discovery; Basel</t>
+        </is>
+      </c>
+      <c r="E96" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2610,17 +3112,22 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Ridgeline Discovery</t>
+          <t>WuXi XDC</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://ridgelinediscovery.com/careers/</t>
+          <t>https://www.wuxixdc.com/careers/</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>CRO drug discovery; Basel</t>
+          <t>CDMO ADC; Basel</t>
+        </is>
+      </c>
+      <c r="E97" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2632,17 +3139,22 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>WuXi XDC</t>
+          <t>T3 Pharmaceuticals</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://www.wuxixdc.com/careers/</t>
+          <t>https://www.t3pharma.com/careers/</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>CDMO ADC; Basel</t>
+          <t>Biotech engineered bacteria; Basel</t>
+        </is>
+      </c>
+      <c r="E98" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2654,17 +3166,22 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>T3 Pharmaceuticals</t>
+          <t>PharmaBiome</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://www.t3pharma.com/careers/</t>
+          <t>https://pharmabio.me/careers/</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Biotech engineered bacteria; Basel</t>
+          <t>Biotech microbiome; Basel</t>
+        </is>
+      </c>
+      <c r="E99" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -2676,17 +3193,22 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PharmaBiome</t>
+          <t>Granite Bio</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://pharmabio.me/careers/</t>
+          <t>https://www.granitebio.com/careers/</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Biotech microbiome; Basel</t>
+          <t>Biotech immunology; Basel</t>
+        </is>
+      </c>
+      <c r="E100" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2698,17 +3220,22 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Granite Bio</t>
+          <t>Stromal Therapeutics</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://www.granitebio.com/careers/</t>
+          <t>https://stromaltx.com/careers/</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Biotech immunology; Basel</t>
+          <t>Biotech tumour stroma; Basel</t>
+        </is>
+      </c>
+      <c r="E101" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -2720,17 +3247,22 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Stromal Therapeutics</t>
+          <t>Straumann Group</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://stromaltx.com/careers/</t>
+          <t>https://www.straumann.com/group/en/discover/career.html</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Biotech tumour stroma; Basel</t>
+          <t>MedTech dental; Basel</t>
+        </is>
+      </c>
+      <c r="E102" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2742,17 +3274,22 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Straumann Group</t>
+          <t>J&amp;J Innovative Medicine</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://www.straumann.com/group/en/discover/career.html</t>
+          <t>https://www.careers.jnj.com/en/jobs/</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>MedTech dental; Basel</t>
+          <t>Pharma; Allschwil (ex-Actelion)</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -2764,17 +3301,22 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>J&amp;J Innovative Medicine</t>
+          <t>Idorsia Pharmaceuticals</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://www.careers.jnj.com/en/jobs/</t>
+          <t>https://careers.idorsia.com/</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Pharma; Allschwil (ex-Actelion)</t>
+          <t>Pharma; Allschwil</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -2786,17 +3328,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Idorsia Pharmaceuticals</t>
+          <t>Basilea Pharmaceutica</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://careers.idorsia.com/</t>
+          <t>https://www.basilea.com/careers</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Pharma; Allschwil</t>
+          <t>Pharma anti-infectives; Allschwil</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2808,17 +3355,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Basilea Pharmaceutica</t>
+          <t>Spexis</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://www.basilea.com/careers</t>
+          <t>https://spexisbio.com/careers/</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Pharma anti-infectives; Allschwil</t>
+          <t>Pharma rare disease; Allschwil</t>
+        </is>
+      </c>
+      <c r="E106" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2830,17 +3382,22 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Spexis</t>
+          <t>Swiss Pharma Contract</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://spexisbio.com/careers/</t>
+          <t>https://swisspharmaco.com/contact/</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Pharma rare disease; Allschwil</t>
+          <t>CRO/CDMO; Allschwil</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2852,17 +3409,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Swiss Pharma Contract</t>
+          <t>CARBOGEN AMCIS</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://swisspharmaco.com/contact/</t>
+          <t>https://www.carbogen-amcis.com/careers/open-positions</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>CRO/CDMO; Allschwil</t>
+          <t>CDMO API &amp; HPAPI; Bubendorf</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2874,17 +3436,22 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>CARBOGEN AMCIS</t>
+          <t>Bachem</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://www.carbogen-amcis.com/careers/open-positions</t>
+          <t>https://careers.bachem.com/search</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>CDMO API &amp; HPAPI; Bubendorf</t>
+          <t>CDMO peptide; Bubendorf (SuccessFactors)</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2896,17 +3463,22 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Bachem</t>
+          <t>Siegfried</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://careers.bachem.com/search</t>
+          <t>https://siegfried.wd103.myworkdayjobs.com/external</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>CDMO peptide; Bubendorf (SuccessFactors)</t>
+          <t>CDMO API; Zofingen (Workday)</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2918,17 +3490,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Siegfried</t>
+          <t>Takeda</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://siegfried.wd103.myworkdayjobs.com/external</t>
+          <t>https://jobs.takeda.com/search-jobs</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>CDMO API; Zofingen (Workday)</t>
+          <t>Pharma; Zurich HQ</t>
+        </is>
+      </c>
+      <c r="E111" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -2940,17 +3517,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Takeda</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://jobs.takeda.com/search-jobs</t>
+          <t>https://careers.abbvie.com/</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Pharma; Zurich HQ</t>
+          <t>Pharma; Zurich</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -2962,17 +3544,22 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>AbbVie</t>
+          <t>Acino</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://careers.abbvie.com/</t>
+          <t>https://acino.swiss/careers/</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Pharma; Zurich</t>
+          <t>Pharma specialty; Zurich</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -2984,17 +3571,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Acino</t>
+          <t>Fosun Pharma</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>https://acino.swiss/careers/</t>
+          <t>https://www.fosunpharma.com/en/careers/</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Pharma specialty; Zurich</t>
+          <t>Pharma; Zurich</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3006,17 +3598,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Fosun Pharma</t>
+          <t>Alvotech</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://www.fosunpharma.com/en/careers/</t>
+          <t>https://www.alvotech.com/about-us/careers</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Pharma; Zurich</t>
+          <t>Pharma biosimilars; Zurich</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3028,17 +3625,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Alvotech</t>
+          <t>MetrioPharm</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://www.alvotech.com/about-us/careers</t>
+          <t>https://www.metriopharm.com/en/about-us/Career.html</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Pharma biosimilars; Zurich</t>
+          <t>Pharma anti-inflammatory; Zurich</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3050,17 +3652,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>MetrioPharm</t>
+          <t>CDR-Life</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://www.metriopharm.com/en/about-us/Career.html</t>
+          <t>https://www.cdr-life.com/careers/</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Pharma anti-inflammatory; Zurich</t>
+          <t>Biotech bispecific ab; Zurich</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3072,17 +3679,22 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>CDR-Life</t>
+          <t>Muvon Therapeutics</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://www.cdr-life.com/careers/</t>
+          <t>https://www.muvon-therapeutics.com/openpositions</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Biotech bispecific ab; Zurich</t>
+          <t>Biotech cell therapy; Zurich</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3094,17 +3706,22 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Muvon Therapeutics</t>
+          <t>Cellvie</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://www.muvon-therapeutics.com/openpositions</t>
+          <t>https://cellvie.bio/careers</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Biotech cell therapy; Zurich</t>
+          <t>Biotech mitochondrial; Zurich</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3116,17 +3733,22 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Cellvie</t>
+          <t>Endogena Therapeutics</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>https://cellvie.bio/careers</t>
+          <t>https://endogena.com/careers/</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Biotech mitochondrial; Zurich</t>
+          <t>Biotech retinal; Zurich</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3138,17 +3760,22 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Endogena Therapeutics</t>
+          <t>Mabylon</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>https://endogena.com/careers/</t>
+          <t>https://mabylon.com/careers/</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Biotech retinal; Zurich</t>
+          <t>Biotech antibodies; Zurich</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3160,17 +3787,22 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Mabylon</t>
+          <t>SYDRA AG</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>https://mabylon.com/careers/</t>
+          <t>https://sydra.io/careers/</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Biotech antibodies; Zurich</t>
+          <t>Biotech AI longevity; Zurich</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3182,17 +3814,22 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SYDRA AG</t>
+          <t>DataHow</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>https://sydra.io/careers/</t>
+          <t>https://datahow.ch/about/careers/</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Biotech AI longevity; Zurich</t>
+          <t>Biotech bioprocess AI; Zurich</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3204,17 +3841,22 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>DataHow</t>
+          <t>QPillars</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>https://datahow.ch/about/careers/</t>
+          <t>https://qpillars.com/careers</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Biotech bioprocess AI; Zurich</t>
+          <t>Pharma quality software; Zurich</t>
+        </is>
+      </c>
+      <c r="E124" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3226,17 +3868,22 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>QPillars</t>
+          <t>MaxWell Biosystems</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>https://qpillars.com/careers</t>
+          <t>https://www.mxwbio.com/careers</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Pharma quality software; Zurich</t>
+          <t>Biotech MEA; Zurich</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3248,17 +3895,22 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>MaxWell Biosystems</t>
+          <t>BC Platforms</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>https://www.mxwbio.com/careers</t>
+          <t>https://careers.bcplatforms.com/</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Biotech MEA; Zurich</t>
+          <t>Biotech genomic platform; Zurich</t>
+        </is>
+      </c>
+      <c r="E126" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3270,17 +3922,22 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>BC Platforms</t>
+          <t>Sequana Medical</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://careers.bcplatforms.com/</t>
+          <t>https://www.sequanamedical.com/open-positions/</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Biotech genomic platform; Zurich</t>
+          <t>MedTech fluid; Zurich</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3292,17 +3949,22 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Sequana Medical</t>
+          <t>Celerion</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://www.sequanamedical.com/open-positions/</t>
+          <t>https://www.celerion.com/careers</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>MedTech fluid; Zurich</t>
+          <t>CRO clinical; Zurich</t>
+        </is>
+      </c>
+      <c r="E128" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3314,17 +3976,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Celerion</t>
+          <t>Molecular Partners</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://www.celerion.com/careers</t>
+          <t>https://www.molecularpartners.com/careers/</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>CRO clinical; Zurich</t>
+          <t>Biotech DARPin; Schlieren</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3336,17 +4003,22 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Molecular Partners</t>
+          <t>Philochem</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>https://www.molecularpartners.com/careers/</t>
+          <t>https://www.philogen.com/en/careers</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Biotech DARPin; Schlieren</t>
+          <t>Biotech drug conjugates; Otelfingen</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3358,17 +4030,22 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Philochem</t>
+          <t>Tandem Therapeutics</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>https://www.philogen.com/en/careers</t>
+          <t>https://jobs.ashbyhq.com/tandem</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Biotech drug conjugates; Otelfingen</t>
+          <t>Biotech ECM/fibrosis; Zurich (Ashby)</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3380,17 +4057,22 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Tandem Therapeutics</t>
+          <t>Amgen</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/tandem</t>
+          <t>https://careers.amgen.com/en/Switzerland</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Biotech ECM/fibrosis; Zurich (Ashby)</t>
+          <t>Pharma; Rotkreuz</t>
+        </is>
+      </c>
+      <c r="E132" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3402,17 +4084,22 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Amgen</t>
+          <t>Roche Diagnostics</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>https://careers.amgen.com/en/Switzerland</t>
+          <t>https://careers.roche.com/global/en/rotkreuz</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Pharma; Rotkreuz</t>
+          <t>Pharma diagnostics; Rotkreuz</t>
+        </is>
+      </c>
+      <c r="E133" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3424,17 +4111,22 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Roche Diagnostics</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>https://careers.roche.com/global/en/rotkreuz</t>
+          <t>https://careers.astrazeneca.com/location/switzerland-jobs/7684/2658434/2</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Pharma diagnostics; Rotkreuz</t>
+          <t>Pharma; Zug</t>
+        </is>
+      </c>
+      <c r="E134" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3446,17 +4138,22 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>AstraZeneca</t>
+          <t>Biogen</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>https://careers.astrazeneca.com/location/switzerland-jobs/7684/2658434/2</t>
+          <t>https://www.biogen.com/careers.html</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Pharma; Zug</t>
+          <t>Biotech neurology; Baar</t>
+        </is>
+      </c>
+      <c r="E135" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3468,17 +4165,22 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Biogen</t>
+          <t>Bristol Myers Squibb</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>https://www.biogen.com/careers.html</t>
+          <t>https://careers.bms.com/</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Biotech neurology; Baar</t>
+          <t>Pharma; Steinhausen</t>
+        </is>
+      </c>
+      <c r="E136" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3490,17 +4192,22 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Bristol Myers Squibb</t>
+          <t>Gilead Sciences</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>https://careers.bms.com/</t>
+          <t>https://jobs.gilead.com/</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Pharma; Steinhausen</t>
+          <t>Pharma antiviral; Zug</t>
+        </is>
+      </c>
+      <c r="E137" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3512,17 +4219,22 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Gilead Sciences</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>https://jobs.gilead.com/</t>
+          <t>https://www.gsk.com/en-gb/careers/</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Pharma antiviral; Zug</t>
+          <t>Pharma oncology unit; Zug</t>
+        </is>
+      </c>
+      <c r="E138" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3534,17 +4246,22 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>https://www.gsk.com/en-gb/careers/</t>
+          <t>https://www.pfizer.com/people/careers</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Pharma oncology unit; Zug</t>
+          <t>Pharma; Zurich/Zug</t>
+        </is>
+      </c>
+      <c r="E139" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3556,17 +4273,22 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Pfizer</t>
+          <t>Galderma</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>https://www.pfizer.com/people/careers</t>
+          <t>https://www.galderma.com/en/careers</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Pharma; Zurich/Zug</t>
+          <t>Pharma dermatology; Zug HQ</t>
+        </is>
+      </c>
+      <c r="E140" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3578,17 +4300,22 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Galderma</t>
+          <t>Blueprint Medicines</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>https://www.galderma.com/en/careers</t>
+          <t>https://job-boards.greenhouse.io/blueprintmedicines</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Pharma dermatology; Zug HQ</t>
+          <t>Biotech precision oncology; Zug (Greenhouse)</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3600,17 +4327,22 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Blueprint Medicines</t>
+          <t>Alnylam</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/blueprintmedicines</t>
+          <t>https://www.alnylam.com/careers</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Biotech precision oncology; Zug (Greenhouse)</t>
+          <t>Biotech RNAi; Zug European HQ</t>
+        </is>
+      </c>
+      <c r="E142" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3622,17 +4354,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Alnylam</t>
+          <t>Nuvation Bio</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>https://www.alnylam.com/careers</t>
+          <t>https://nuvationbio.com/careers/</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Biotech RNAi; Zug European HQ</t>
+          <t>Biotech oncology; Zug</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3644,17 +4381,22 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Nuvation Bio</t>
+          <t>Apellis</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>https://nuvationbio.com/careers/</t>
+          <t>https://apellis.com/careers/</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Biotech oncology; Zug</t>
+          <t>Biotech complement; Zug</t>
+        </is>
+      </c>
+      <c r="E144" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3666,17 +4408,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Apellis</t>
+          <t>Immunocore</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>https://apellis.com/careers/</t>
+          <t>https://jobs.ashbyhq.com/immunocore</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Biotech complement; Zug</t>
+          <t>Biotech ImmTAX; Zug (Ashby)</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3688,17 +4435,22 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Immunocore</t>
+          <t>PSI CRO</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/immunocore</t>
+          <t>https://psi-cro.com/careers/</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Biotech ImmTAX; Zug (Ashby)</t>
+          <t>CRO full-service; Zug</t>
+        </is>
+      </c>
+      <c r="E146" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3710,17 +4462,22 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PSI CRO</t>
+          <t>PolyPeptide Group</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>https://psi-cro.com/careers/</t>
+          <t>https://www.polypeptide.com/careers</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>CRO full-service; Zug</t>
+          <t>CDMO peptide; Zug</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3732,17 +4489,22 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PolyPeptide Group</t>
+          <t>Recipharm</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>https://www.polypeptide.com/careers</t>
+          <t>https://www.recipharm.com/join-us/</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>CDMO peptide; Zug</t>
+          <t>CDMO drug product; Zug</t>
+        </is>
+      </c>
+      <c r="E148" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3754,17 +4516,22 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Recipharm</t>
+          <t>CSL Behring</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>https://www.recipharm.com/join-us/</t>
+          <t>https://www.csl.com/careers</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>CDMO drug product; Zug</t>
+          <t>Pharma plasma-derived; Bern</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3776,17 +4543,22 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>CSL Behring</t>
+          <t>AlveoliX</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>https://www.csl.com/careers</t>
+          <t>https://www.alveolix.com/about/</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Pharma plasma-derived; Bern</t>
+          <t>Biotech lung-on-chip; Bern</t>
+        </is>
+      </c>
+      <c r="E150" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3798,17 +4570,22 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>AlveoliX</t>
+          <t>CellnTec</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>https://www.alveolix.com/about/</t>
+          <t>https://cellntec.com/careers/</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Biotech lung-on-chip; Bern</t>
+          <t>Biotech epithelial cell culture; Bern</t>
+        </is>
+      </c>
+      <c r="E151" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3820,17 +4597,22 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>CellnTec</t>
+          <t>Ypsomed</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>https://cellntec.com/careers/</t>
+          <t>https://www.ypsomed.com/en/careers.html</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Biotech epithelial cell culture; Bern</t>
+          <t>MedTech drug delivery; Burgdorf</t>
+        </is>
+      </c>
+      <c r="E152" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3842,17 +4624,22 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Ypsomed</t>
+          <t>Ferring Pharmaceuticals</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>https://www.ypsomed.com/en/careers.html</t>
+          <t>https://www.ferring.com/careers/</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>MedTech drug delivery; Burgdorf</t>
+          <t>Pharma reproductive health; St-Prex</t>
+        </is>
+      </c>
+      <c r="E153" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3864,17 +4651,22 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Ferring Pharmaceuticals</t>
+          <t>Debiopharm</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>https://www.ferring.com/careers/</t>
+          <t>https://apply.workable.com/debiopharm/</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Pharma reproductive health; St-Prex</t>
+          <t>Pharma oncology; Lausanne (Workable)</t>
+        </is>
+      </c>
+      <c r="E154" s="10" t="inlineStr">
+        <is>
+          <t>Skip</t>
         </is>
       </c>
     </row>
@@ -3886,17 +4678,22 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Debiopharm</t>
+          <t>AC Immune</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/debiopharm/</t>
+          <t>https://www.acimmune.com/careers/</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Pharma oncology; Lausanne (Workable)</t>
+          <t>Biotech neurodegeneration; Lausanne</t>
+        </is>
+      </c>
+      <c r="E155" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3908,17 +4705,22 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>AC Immune</t>
+          <t>HAYA Therapeutics</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>https://www.acimmune.com/careers/</t>
+          <t>https://www.hayatx.com/careers</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Biotech neurodegeneration; Lausanne</t>
+          <t>Biotech lncRNA; Lausanne</t>
+        </is>
+      </c>
+      <c r="E156" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3930,17 +4732,22 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>HAYA Therapeutics</t>
+          <t>Oculis</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>https://www.hayatx.com/careers</t>
+          <t>https://oculis.com/jobs/</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Biotech lncRNA; Lausanne</t>
+          <t>Biotech eye disease; Lausanne</t>
+        </is>
+      </c>
+      <c r="E157" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3952,17 +4759,22 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Oculis</t>
+          <t>AB2 Bio</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>https://oculis.com/jobs/</t>
+          <t>http://www.ab2bio.com/en/careers.32.html</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Biotech eye disease; Lausanne</t>
+          <t>Biotech IL-18; Lausanne</t>
+        </is>
+      </c>
+      <c r="E158" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3974,17 +4786,22 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>AB2 Bio</t>
+          <t>Ichnos Sciences</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>http://www.ab2bio.com/en/careers.32.html</t>
+          <t>https://iginnovate.com/careers/</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Biotech IL-18; Lausanne</t>
+          <t>Biotech bispecific ab; Lausanne (IGI)</t>
+        </is>
+      </c>
+      <c r="E159" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -3996,17 +4813,22 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Ichnos Sciences</t>
+          <t>Opna Bio</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>https://iginnovate.com/careers/</t>
+          <t>https://www.opnabio.com/careers/</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Biotech bispecific ab; Lausanne (IGI)</t>
+          <t>Biotech oncology; Epalinges</t>
+        </is>
+      </c>
+      <c r="E160" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4018,17 +4840,22 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Opna Bio</t>
+          <t>Onward Therapeutics</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>https://www.opnabio.com/careers/</t>
+          <t>https://www.onwardtherapeutics.com/careers/</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
           <t>Biotech oncology; Epalinges</t>
+        </is>
+      </c>
+      <c r="E161" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4040,17 +4867,22 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Onward Therapeutics</t>
+          <t>RS Research</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>https://www.onwardtherapeutics.com/careers/</t>
+          <t>https://rsresearch.net/careers/</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Biotech oncology; Epalinges</t>
+          <t>CRO clinical; Lausanne</t>
+        </is>
+      </c>
+      <c r="E162" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
@@ -4062,39 +4894,22 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>RS Research</t>
+          <t>Novostia</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>https://rsresearch.net/careers/</t>
+          <t>https://www.novostia.com/careers</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>CRO clinical; Lausanne</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>Switzerland</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>Novostia</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>https://www.novostia.com/careers</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
           <t>MedTech cardiac; Lausanne</t>
+        </is>
+      </c>
+      <c r="E163" s="9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add 84 new Swiss company career pages to scraper list
Adds 84 Swiss biotech/pharma/CRO/specialty-chem companies to
European_Job_Search_Websites.xlsx (199 Switzerland entries total).

New _OVERRIDES in _registry.py:
- jobs.syngenta.com: SmartRecruiters keyword search URL
- iabxas.fa.ocs.oraclecloud.com: Oracle Cloud HCM for Solvias
- join.com/companies/virometix: join.com ATS job-link pattern
- baselaunch.ch: skip (incubator, no scrapeable listings)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/European_Job_Search_Websites.xlsx
+++ b/European_Job_Search_Websites.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E165"/>
+  <dimension ref="A1:E249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4964,6 +4964,2274 @@
         </is>
       </c>
       <c r="E165" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>BaseLaunch</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://baselaunch.ch/</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Major Basel biotech incubator/accelerator; 30+ portfolio ventures; partners incl. Roche, J&amp;J, AbbVie, Pfizer</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Araris Biotech</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://www.ararisbiotech.com/</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>ADC linker/conjugation platform; acquired by Taiho Pharmaceutical 2025</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Sika</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://www.sika.com/en/careers.html</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Specialty chemicals for construction and industry; polymers, mortars, sealants; Baar HQ</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Cerbios-Pharma</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://www.cerbios.ch/careers</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>CDMO for HPAPIs, ADCs, and biologics; Barbengo</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Polyneuron Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://www.polyneuron.com/</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Glycopolymer-based therapeutics for autoimmune diseases; carbohydrate chemistry; Basel</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Nouscom</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://nouscom.com/</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Immuno-oncology; viral-vectored neoantigen vaccines; Basel R&amp;D/manufacturing</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Vaderis Therapeutics</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://www.vaderis.com/</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Clinical-stage; rare vascular malformation diseases; small-molecule focus; Basel</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Baliopharm</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://www.baliopharm.com/</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Chronic liver disease, immune-mediated inflammatory disease, and cancer; Basel</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Amphilix</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://www.amphilix.com/</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Next-gen radioligand therapy; proprietary 3D linker platform; lead AMX-0053 colorectal cancer; Basel</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Allegria Therapeutics</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://www.allegriatx.com/</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Mast-cell-modulating therapeutics for allergy and inflammatory disease; founded 2023; Basel</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>NXI Therapeutics</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://www.nxi-tx.com/</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Clinical-stage oncology biotech; Basel</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>FimmCyte</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://www.fimmcyte.com/</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Autoimmune disease therapeutics; Basel</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Myria Biosciences</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://www.myriabiosciences.com/</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Early-stage biotech; Basel</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Inofea</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://www.inofea.com/</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Protein engineering and conjugate technologies; Basel</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Evotec</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://careers.evotec.com/</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Integrated drug discovery CRO; INDiGO, ADC, biologics platforms; small Basel office</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Orion Corporation Switzerland</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://www.orion.fi/en/careers/</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Finnish pharma Swiss affiliate; some R&amp;D/drug discovery roles; Basel</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Friedrich Miescher Institute (FMI)</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://www.fmi.ch/career/</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Basic biomedical research; Novartis-sponsored; strong feeder for industry hires; Basel</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Vicebio</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://www.vicebio.com/careers</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Vaccine development for respiratory viruses; Basel presence via London HQ</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>AmRNA</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://www.amrna.ch/</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>RNA reagents, gene synthesis, and research services; preclinical development support; Basel</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Syngenta</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://jobs.syngenta.com/</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>World-leading agrochemistry; active ingredient discovery; Stein AG research site; Basel</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Corteva</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://www.corteva.com/careers</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Agrochemistry spun off DowDuPont; Swiss hub Basel/Schweizerhalle</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>BASF Switzerland</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://www.basf.com/global/en/careers</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Specialty chemicals, agrochem, pharma intermediates; Basel/Kaisten sites</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>CSL Vifor</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://careers.csl.com/</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Iron deficiency and nephrology; CSL subsidiary; Bern HQ</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Senn Chemicals</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://www.sennchem.com/contact-news/career</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Custom GMP synthesis of peptides, amino acid derivatives, and small molecules; Dielsdorf</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Ems-Chemie</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://www.emsgroup.com/en/career/</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>High-performance polyamides, adhesives, and polymer chemistry; Domat/Ems</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Dottikon Exclusive Synthesis</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://dottikon.com/en/jobs-careers/</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Custom synthesis and exclusive manufacture of fine chemicals and APIs; safety-critical reactions; Dottikon</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>ADC Therapeutics</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://adctherapeutics.com/careers/</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>ADCs for hematological and solid cancers; Zynlonta approved for DLBCL; Epalinges</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Novigenix</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://www.novigenix.com/</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Blood-based early cancer detection diagnostics; Epalinges</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Mymetics</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://www.mymetics.com/</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Virosome-based vaccines; malaria, RSV, HSV-2; Epalinges</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Addex Therapeutics</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://www.addextherapeutics.com/en/about-us/careers/</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Small-molecule allosteric modulators for CNS and neurological disorders; Geneva</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>GeNeuro</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://geneuro.ch/en/contact/</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Autoimmune and neurodegeneration antibodies targeting HERV-related mechanisms; Geneva</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>AMAL Therapeutics</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://www.amaltherapeutics.com/careers</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Therapeutic cancer vaccines KISIMA platform; part of Boehringer Ingelheim since 2019; Geneva</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Relief Therapeutics</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://www.relieftherapeutics.com/careers</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Specialty pharma; rare diseases; aviptadil and partnership pipeline; Geneva</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Oncodesign Services</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://www.oncodesign-services.com/careers/</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Integrated preclinical/medicinal chemistry CRO in oncology, autoimmune, infection; DMPK; Geneva</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>dsm-firmenich</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://www.dsm-firmenich.com/corporate/careers.html</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Fragrance, flavour, nutrition and health; large chemistry/biotech footprint; Kaiseraugst/Vernier sites</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Mettler-Toledo</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://careers.mt.com/</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Precision analytical instruments for chemistry labs; pH, titration, thermal analysis; Greifensee</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Solvias</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://iabxas.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/jobs</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>CRO for CMC analytics, API development, and method development; supports med-chem projects; Kaiseraugst</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Isomorphic Labs</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://www.isomorphiclabs.com/job-openings</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Google DeepMind/Alphabet drug-discovery arm; AI-first drug design using AlphaFold3; Lausanne computational team</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Amazentis</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://www.amazentis.com/careers</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Urolithin A Mitopure - mitochondrial health/longevity; EPFL spin-off; Lausanne</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Asceneuron</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://www.asceneuron.com/careers</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Small-molecule O-GlcNAcase inhibitors for tauopathies PSP Alzheimer; clinical-stage; Lausanne</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Anokion</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://www.anokion.com/careers</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Autoimmune disease tolerance platform MS celiac T1 diabetes; EPFL spin-off; Lausanne</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Orbis Medicines</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://orbismedicines.com/careers/</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>AI-enabled oral macrocycle drug design; Prof Heinis EPFL lab origin; Lausanne</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Leman Biotech</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://www.lemanbio.com/</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Metabolic cancer immunotherapies and CAR-T; EPFL spin-off; Lausanne</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Biodelphis Therapeutics</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://biodelphistx.com/</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Next-generation protease inhibitors for cancer, autoimmune, and bone diseases; EPFL spin-off; Lausanne</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>HemostOD</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://www.hemostod.com/</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>In vitro human platelets platform; EPFL Innovation Park; Lausanne</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Limula</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://www.limula.ch/careers</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Closed/automated CAR-T and cell therapy manufacturing platform; Lausanne</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Mindmaze</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://www.mindmaze.com/careers/</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Neurotech - digital therapeutics for stroke and neurological injury recovery; Lausanne</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Incyte Biosciences International</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://careers.incyte.com/jobs</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Global biopharma in oncology, inflammation and autoimmunity; Swiss site in Morges</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>CordenPharma</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://cordenpharma.com/careers/opportunities/</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Full-service CDMO for APIs, peptides/oligos, LNPs, drug product; Muttenz BL + Basel HQ</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Clariant</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://www.clariant.com/en/Careers</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Specialty chemicals - catalysts, care chemicals, natural resources; HQ Muttenz</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>CSEM</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://www.csem.ch/careers</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Applied R&amp;D - surface chemistry, microfluidics, sensors, digital health devices; Neuchatel</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Omya</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://www.omya.com/en/careers</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Industrial minerals CaCO3 dolomite for pharma excipients, paper, plastics, paints; Oftringen</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Santhera Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://www.santhera.com/careers</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Rare-disease small-molecule development and commercialization; HQ Pratteln BL</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>SI Group</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://www.siigroup.com/careers</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Performance additives for polymers - antioxidants, UV stabilizers; HQ Pratteln</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Sicpa</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://www.sicpa.com/careers</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Security inks and authentication technologies; surface chemistry/ink formulation; Prilly</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Sophia Genetics</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://www.sophiagenetics.com/careers/</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>AI platform for genomic data analysis; personalized medicine for cancer and genetic diseases; Rolle</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Neurimmune</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://www.neurimmune.com/careers</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Antibody therapeutics from human immune memory; neurodegeneration and cardiovascular; Schlieren</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>InSphero</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://insphero.com/careers/</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>3D in vitro microtissue models and services for drug discovery and safety testing; Schlieren</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Virometix</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://join.com/companies/virometix</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Clinical-stage; synthetic vaccines for infectious diseases and cancer; Schlieren</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>DiNAQOR</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://www.dinaqor.com/about-us/careers/</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Gene therapy platform; develops and manufactures gene therapies; Schlieren</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>CUTISS</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://cutiss.swiss/career/</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Automated personalized skin tissue therapeutics for reconstructive surgery; Schlieren</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>EraCal Therapeutics</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://eracal.ch/</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Small-molecule appetite suppressants for anti-obesity; NCE from in-vivo discovery platform; Schlieren</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Anjarium Biosciences</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://www.anjarium.com/careers</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Non-viral gene delivery Hybridosome platform; engineered extracellular vesicles; Schlieren</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Topadur Pharma</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://topadur.com/</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Small-molecule DualTOP platform targeting microcirculation and regeneration; Schlieren</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Oncobit</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://www.oncobit.com/careers</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Precision oncology - ctDNA diagnostics and AI-based cancer monitoring; Schlieren</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Synergene Biotech</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://www.synergene.ch/</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Molecular biology services; UZH spin-off 2001; Schlieren</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Buehlmann Laboratories</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://www.buhlmannlabs.ch/careers/</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>In vitro diagnostics - immunology and gastroenterology assays; Schoenenbuch</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Biosynth</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://www.biosynth.com/careers</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Fine chemicals, custom synthesis, complex carbohydrates, nucleotides, peptides, natural products; Staad</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Lunaphore</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://bio-techne.com/careers</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Spatial biology/automated immunohistochemistry; acquired by Bio-Techne 2024; Tolochenaz</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Givaudan</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://careers.givaudan.com/</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>World-leading fragrance and flavour house; organic chemistry, biocatalysis, natural product chemistry; Vernier</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Paul Scherrer Institute (PSI)</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://www.psi.ch/en/hr/job-opportunities</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Largest Swiss research institute; SwissFEL/SLS for structural biology; radiopharmaceuticals; Villigen</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>leadxpro</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>https://careers.leadxpro.com/</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Structure-based drug design SBDD CRO; AI and drug discovery; Villigen</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Polpharma Biologics</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>https://careers.polpharma.com/</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Biosimilars manufacturing; Visp VS site</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Welmedis AG</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>https://www.welmedis.com/</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Organic/medicinal chemistry contract research and project-based drug discovery; Waedenswil</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>GlycoEra</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>https://www.glycoera.com/careers-2/</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Glycoengineered biologics for selective degradation of immune targets; autoimmune/inflammatory diseases; Waedenswil</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Numab Therapeutics</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://www.numab.com/careers/</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Multispecific antibody therapeutics inflammation and cancer; MATCH and lambda-Cap platforms; Waedenswil</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>MoonLake Immunotherapeutics</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>https://moonlaketx.com/careers/</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Nanobody-based therapies for inflammatory skin and joint diseases; public biotech; Zug</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>CRISPR Therapeutics</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>https://crisprtx.com/careers</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>CRISPR/Cas9 gene-based medicines; Casgevy sickle cell approved 2023; oncology/autoimmune/diabetes pipeline; Zug</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Centenara Labs</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>https://www.centenara.com/</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Longevity/healthy-aging therapeutics; formerly Rejuveron; creates and invests in new drug programs; Zurich</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Adularia</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>https://adularia.ch/</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Precision cancer immunotherapy; pivoted to small-molecule targeting; Zurich</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>TwinEdge Bioscience</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>https://www.twinedge.bio/</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Digital twins for oncology drug discovery and development; computational biology + AI; Zurich</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Ai.Qimia</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://www.aiqimia.com/</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Physics-based AI and quantum simulation for synthesis prediction in process chemistry; Zurich</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Rejuveron Life Sciences</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>https://www.rejuveron.com/careers</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Longevity/age-related disease biotech platform; portfolio of multiple spin-outs; Zurich</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>AMYRA</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>https://www.amyra.ch/</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Enzyme therapeutics for celiac disease and non-celiac gluten sensitivity; Switzerland</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
         <is>
           <t>Active</t>
         </is>

</xml_diff>